<commit_message>
Atualização de documentação restante de S04
</commit_message>
<xml_diff>
--- a/01-artefactos-de-gestao/01.04-backlog-de-projeto/m1-backlog-projeto-v01.xlsx
+++ b/01-artefactos-de-gestao/01.04-backlog-de-projeto/m1-backlog-projeto-v01.xlsx
@@ -6016,9 +6016,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100293B981485C9E24DAE651C97D9FBC267" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="81e1889baf096e0f1fabc7e628f510b3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="32f33a6e-f018-4796-a6d6-b8c30f0661e9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4b8b816b6954550eb9ea5c593f5cc868" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100293B981485C9E24DAE651C97D9FBC267" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="73cbee31f6114801cea13732a9ec5387">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="32f33a6e-f018-4796-a6d6-b8c30f0661e9" xmlns:ns3="59ec22bb-74c1-4c3c-af96-122e757b18d2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cc47ff3526632fc7ff348bab4cf07ac" ns2:_="" ns3:_="">
     <xsd:import namespace="32f33a6e-f018-4796-a6d6-b8c30f0661e9"/>
+    <xsd:import namespace="59ec22bb-74c1-4c3c-af96-122e757b18d2"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -6028,6 +6029,11 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -6052,6 +6058,43 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1374c586-51ca-419d-b13a-551147e70874" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="59ec22bb-74c1-4c3c-af96-122e757b18d2" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{281605ea-d3cc-4310-8c97-aa0e64c9f496}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="59ec22bb-74c1-4c3c-af96-122e757b18d2">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -6164,26 +6207,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="59ec22bb-74c1-4c3c-af96-122e757b18d2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="32f33a6e-f018-4796-a6d6-b8c30f0661e9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94B8A81E-A4DB-4E62-AF2B-35FDE0E6F1AA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="32f33a6e-f018-4796-a6d6-b8c30f0661e9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{919CA136-9F07-4A16-91BD-77C2113B40C3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>